<commit_message>
EPBDS-16529 Index the ternary whose lookup is written as its last part
A condition such as "isEmpty(code) ? fallback : contains(codes, code)" says the
same as the form the index already understood, only the other way round, and was
evaluated row by row. The test now points at one of the two parts: whichever of
them is the lookup runs against the index, and the other one answers the whole
condition.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-16529_DecisionTable_TernaryCondition.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-16529_DecisionTable_TernaryCondition.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J47"/>
+  <dimension ref="B2:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="2" max="2"/>
@@ -1126,6 +1126,11 @@
           <t>Result</t>
         </is>
       </c>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>Test selectByCodeReversed selectByCodeReversedTest</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="2" t="inlineStr">
@@ -1138,6 +1143,21 @@
           <t>Foo</t>
         </is>
       </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="2" t="inlineStr">
@@ -1148,6 +1168,21 @@
       <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Bar</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Fallback</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>
@@ -1156,6 +1191,364 @@
       <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Any</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="H50" s="2" t="n"/>
+      <c r="I50" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>Rules String selectByCodeReversed(String code, Boolean fallback)</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>isEmpty(code) ? fallback : contains(codes, code)</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>Test compareReversed compareReversedTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>foo,baz</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Foo</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Fallback</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="H60" s="2" t="n"/>
+      <c r="I60" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="H61" s="2" t="n"/>
+      <c r="I61" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>same</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>Rules String selectByCodeReversedNotIndexed(String code, Boolean fallback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>(isEmpty(code) ? fallback : contains(codes, code)) or false</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>String[] codes</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>foo,baz</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Foo</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="1" t="inlineStr">
+        <is>
+          <t>Method String compareReversed(String code, Boolean fallback)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>return selectByCodeReversed(code, fallback) == selectByCodeReversedNotIndexed(code, fallback) ? "same" : "different";</t>
         </is>
       </c>
     </row>

</xml_diff>